<commit_message>
Actualización automática de noticias - 2026-09-15
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Impactante video de una joven que se lanzó por un tobogán en Cocorná, Antioquia: la adolescente quedó inconsciente en la piscina</t>
+          <t>Una empresa digital de aseo de hogares y oficinas le ha ido ganando terreno a la tradicional Casa Limpia</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,12 +486,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,12 +501,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/09/14/impactante-video-de-una-joven-que-se-lanzo-por-un-tobogan-en-cocorna-antioquia-la-adolescente-quedo-inconsciente-en-la-piscina/</t>
+          <t>https://www.las2orillas.co/una-empresa-digital-de-aseo-de-hogares-y-oficinas-le-ha-ido-ganando-terreno-a-la-tradicional-casa-limpia/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Las imágenes difundidas en redes sociales muestran el instante en que la usuaria llegó al agua y la reacción de varias personas para socorrerla</t>
+          <t>Hogarú nació para responder a las necesidades de jóvenes que han cambiado la relación laboral directa con empleadas domésticasEl artículoUna empresa digital de aseo de hogares y oficinas le ha ido ganando terreno a la tradicional Casa Limpiafue...</t>
         </is>
       </c>
     </row>
@@ -518,12 +518,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Una empresa digital de aseo de hogares y oficinas le ha ido ganando terreno a la tradicional Casa Limpia</t>
+          <t>Impactante video de una joven que se lanzó por un tobogán en Cocorná, Antioquia: la adolescente quedó inconsciente en la piscina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -533,12 +533,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -548,12 +548,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/una-empresa-digital-de-aseo-de-hogares-y-oficinas-le-ha-ido-ganando-terreno-a-la-tradicional-casa-limpia/</t>
+          <t>https://www.infobae.com/colombia/2026/09/14/impactante-video-de-una-joven-que-se-lanzo-por-un-tobogan-en-cocorna-antioquia-la-adolescente-quedo-inconsciente-en-la-piscina/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Hogarú nació para responder a las necesidades de jóvenes que han cambiado la relación laboral directa con empleadas domésticasEl artículoUna empresa digital de aseo de hogares y oficinas le ha ido ganando terreno a la tradicional Casa Limpiafue...</t>
+          <t>Las imágenes difundidas en redes sociales muestran el instante en que la usuaria llegó al agua y la reacción de varias personas para socorrerla</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-09-16
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Una empresa digital de aseo de hogares y oficinas le ha ido ganando terreno a la tradicional Casa Limpia</t>
+          <t>Familia busca a Hever Stiven Muñoz Giraldo, joven desaparecido en la vereda Chembe de Ibagué desde el 8 de septiembre</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,12 +486,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Ibagué</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,14 +501,10 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/una-empresa-digital-de-aseo-de-hogares-y-oficinas-le-ha-ido-ganando-terreno-a-la-tradicional-casa-limpia/</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Hogarú nació para responder a las necesidades de jóvenes que han cambiado la relación laboral directa con empleadas domésticasEl artículoUna empresa digital de aseo de hogares y oficinas le ha ido ganando terreno a la tradicional Casa Limpiafue...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/desaparicion-de-hever-stiven-munoz-giraldo-en-ibague-datos-clave-y-como-ayudar-PP5304535A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-09-22
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Joven de 20 años fue asesinado durante una riña cerca del estadio Armando Maestre en Valledupar</t>
+          <t>Un dirigente empresarial y político samario cuñado del influyente Joaquín Gutiérrez será el presidente de Coljuegos</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,12 +486,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,30 +501,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/valledupar-detalles-del-asesinato-de-keiner-acuna-y-captura-de-gonzalo-palacio-cujia-PP5309154A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>https://www.las2orillas.co/un-dirigente-empresarial-y-politico-samario-cunado-del-influyente-joaquin-gutierrez-sera-el-presidente-de-coljuegos/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Jaime Vives Pinedo llega a uno de los cargos bien remunerados en un momento en que el sector está al alza y mueve un presupuesto anual de $ 1.5 billonesEl artículoUn dirigente empresarial y político samario cuñado del influyente Joaquín Gutiérrez...</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jóvenes con machetes se subieron a una ‘chiva rumbera’ y generaron pánico en Ibagué: autoridades investigan lo ocurrido</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,22 +538,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ibagué</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/09/21/jovenes-con-machetes-se-subieron-a-una-chiva-rumbera-y-generaron-panico-en-ibague-autoridades-investigan-lo-ocurrido/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>La hipótesis preliminar apunta a un conflicto entre jóvenes de distintas comunas, algunos posiblemente menores de edad</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -561,12 +565,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Un dirigente empresarial y político samario cuñado del influyente Joaquín Gutiérrez será el presidente de Coljuegos</t>
+          <t>Joven de 20 años fue asesinado durante una riña cerca del estadio Armando Maestre en Valledupar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -576,12 +580,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -591,14 +595,10 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/un-dirigente-empresarial-y-politico-samario-cunado-del-influyente-joaquin-gutierrez-sera-el-presidente-de-coljuegos/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Jaime Vives Pinedo llega a uno de los cargos bien remunerados en un momento en que el sector está al alza y mueve un presupuesto anual de $ 1.5 billonesEl artículoUn dirigente empresarial y político samario cuñado del influyente Joaquín Gutiérrez...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/valledupar-detalles-del-asesinato-de-keiner-acuna-y-captura-de-gonzalo-palacio-cujia-PP5309154A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Jóvenes con machetes se subieron a una ‘chiva rumbera’ y generaron pánico en Ibagué: autoridades investigan lo ocurrido</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Ibagué</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.infobae.com/colombia/2026/09/21/jovenes-con-machetes-se-subieron-a-una-chiva-rumbera-y-generaron-panico-en-ibague-autoridades-investigan-lo-ocurrido/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>La hipótesis preliminar apunta a un conflicto entre jóvenes de distintas comunas, algunos posiblemente menores de edad</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-09-25
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,27 +466,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Por muerte de Donovan Balanta Paz en Ciudad Bolívar, Policía anunció investigación disciplinaria y suspendió a siete uniformados</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -501,12 +501,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/09/23/por-muerte-de-donovan-balanta-paz-en-ciudad-bolivar-policia-anuncio-investigacion-disciplinaria-y-suspendio-a-siete-uniformados/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>El caso se presentó en el sector de Caracolí, un punto limítrofe entre el sur de Bogotá y el vecino municipio de Soacha, en Cundinamarca. La familia del joven de 34 años pide justicia</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -518,22 +518,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Por muerte de Donovan Balanta Paz en Ciudad Bolívar, Policía anunció investigación disciplinaria y suspendió a siete uniformados</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -548,12 +548,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/09/23/por-muerte-de-donovan-balanta-paz-en-ciudad-bolivar-policia-anuncio-investigacion-disciplinaria-y-suspendio-a-siete-uniformados/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>El caso se presentó en el sector de Caracolí, un punto limítrofe entre el sur de Bogotá y el vecino municipio de Soacha, en Cundinamarca. La familia del joven de 34 años pide justicia</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-02
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,22 +466,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Colombia está entre los países en que las personas se pensionan más jóvenes, según la Ocde: esta es la comparación con otros lugares</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,22 +491,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/10/01/colombia-esta-entre-los-paises-en-que-las-personas-se-pensionan-mas-jovenes-segun-la-ocde-esta-es-la-comparacion-con-otros-lugares/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>En el país las mujeres pueden acceder a la prestación desde los 57 años y los hombres desde los 62, frente a las referencias internacionales de 63,9 y 64,7 registradas en 2024 entre los países analizados</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -518,12 +518,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Uno de cada cuatro jovenes de 18 a 24 anos en colombia es 'nini', no estudia ni trabaja, el doble de la ocde</t>
+          <t>Colombia está entre los países en que las personas se pensionan más jóvenes, según la Ocde: esta es la comparación con otros lugares</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Portafolio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -548,10 +548,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.portafolio.co/economia/uno-de-cada-cuatro-jovenes-de-18-a-24-anos-en-colombia-es-nini-no-estudia-ni-trabaja-el-doble-de-la-ocde-503651</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>https://www.infobae.com/colombia/2026/10/01/colombia-esta-entre-los-paises-en-que-las-personas-se-pensionan-mas-jovenes-segun-la-ocde-esta-es-la-comparacion-con-otros-lugares/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>En el país las mujeres pueden acceder a la prestación desde los 57 años y los hombres desde los 62, frente a las referencias internacionales de 63,9 y 64,7 registradas en 2024 entre los países analizados</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -561,17 +565,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Uno de cada cuatro jovenes de 18 a 24 anos en colombia es 'nini', no estudia ni trabaja, el doble de la ocde</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Portafolio</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -581,24 +585,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
-        </is>
-      </c>
+          <t>https://www.portafolio.co/economia/uno-de-cada-cuatro-jovenes-de-18-a-24-anos-en-colombia-es-nini-no-estudia-ni-trabaja-el-doble-de-la-ocde-503651</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-04
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I235"/>
+  <dimension ref="A1:I233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,22 +466,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Asesinan a joven líder social en Tibú, Norte de Santander: el caso de Magnely Pallares Franco y el conflicto en Catatumbo</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,20 +491,24 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cúcuta</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/magnely-pallares-franco-lider-social-asesinado-en-tibu-norte-de-santander-que-paso-PP5320707A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,17 +518,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Asesinan a joven líder social en Tibú, Norte de Santander: el caso de Magnely Pallares Franco y el conflicto en Catatumbo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,24 +538,20 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cúcuta</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/magnely-pallares-franco-lider-social-asesinado-en-tibu-norte-de-santander-que-paso-PP5320707A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7596,12 +7596,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Voluntariado transformador: unidad de autocuidado para habitantes de calle en el Voto Nacional estrena ludoteca</t>
+          <t>Abierta convocatoria para la Escuela Distrital de Emprendimiento para jóvenes en Engativá</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -7631,29 +7631,29 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#364408dd32</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#248fcdb8a0</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>• 40 personas, entre voluntarios de empresas y habitantes de calle, unieron esfuerzos para adecuar un espacio que estimula el conocimiento y pone a volar a la imaginación. • Esta acción se enmarca en la estrategia ‘Más manos por Bogotá’, programa de...</t>
+          <t>• El Distrito abre la convocatoria para 50 jóvenes entre 18 y 28 años, que cuentan con un emprendimiento en marcha y buscan fortalecer sus capacidades para hacerlo crecer y consolidarlo. • La formación se realizará de manera presencial en la Casa de...</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Abierta convocatoria para la Escuela Distrital de Emprendimiento para jóvenes en Engativá</t>
+          <t>Miles de jóvenes se toman Bogotá: Prosperidad Social acompaña el Festival Nacional de la Juventud</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -7678,91 +7678,91 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#248fcdb8a0</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/miles-de-jovenes-se-toman-bogota-prosperidad-social-acompana-el-festival-nacional-de-la-juventud/</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>• El Distrito abre la convocatoria para 50 jóvenes entre 18 y 28 años, que cuentan con un emprendimiento en marcha y buscan fortalecer sus capacidades para hacerlo crecer y consolidarlo. • La formación se realizará de manera presencial en la Casa de...</t>
+          <t>Más de 4.000 jóvenes de todo el país se reúnen del 24 al 26 de abril en la sede Aduanilla de Paiba de la Universidad Distrital</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Miles de jóvenes se toman Bogotá: Prosperidad Social acompaña el Festival Nacional de la Juventud</t>
+          <t>El tío comunista de Paloma Valencia, la oveja negra que incomodó a su familia conservadora</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Popayán</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/miles-de-jovenes-se-toman-bogota-prosperidad-social-acompana-el-festival-nacional-de-la-juventud/</t>
+          <t>https://www.las2orillas.co/el-tio-comunista-de-paloma-valencia-la-oveja-negra-que-incomodo-a-su-familia-conservadora/</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Más de 4.000 jóvenes de todo el país se reúnen del 24 al 26 de abril en la sede Aduanilla de Paiba de la Universidad Distrital</t>
+          <t>Álvaro Pío Valencia, hermano del expresidente Guillermo León, conoció de joven al papá de Iván Cepeda en Popayán e influyó para que él fuera un consagrado ComunistaEl artículoEl tío comunista de Paloma Valencia, la oveja negra que incomodó a su...</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>El tío comunista de Paloma Valencia, la oveja negra que incomodó a su familia conservadora</t>
+          <t>Masacre en Mocoa: asesinaron a cinco jóvenes en zona boscosa</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Popayán</t>
+          <t>Mocoa</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -7772,12 +7772,12 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/el-tio-comunista-de-paloma-valencia-la-oveja-negra-que-incomodo-a-su-familia-conservadora/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/masacre-en-mocoa-asesinaron-a-cinco-jovenes-en-zona-boscosa/</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Álvaro Pío Valencia, hermano del expresidente Guillermo León, conoció de joven al papá de Iván Cepeda en Popayán e influyó para que él fuera un consagrado ComunistaEl artículoEl tío comunista de Paloma Valencia, la oveja negra que incomodó a su...</t>
+          <t>Cinco hombres fueron asesinados en Mocoa. El hecho se dio después de que se difundió un panfleto amenazante.</t>
         </is>
       </c>
     </row>
@@ -7789,7 +7789,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Masacre en Mocoa: asesinaron a cinco jóvenes en zona boscosa</t>
+          <t>Patinador de 14 años de la Liga Vallecaucana murió durante un entrenamiento: esto se sabe</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Mocoa</t>
+          <t>Popayán</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -7819,24 +7819,24 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/masacre-en-mocoa-asesinaron-a-cinco-jovenes-en-zona-boscosa/</t>
+          <t>https://www.elespectador.com/colombia/cali/muere-joven-patinador-en-cali-tras-accidente-durante-entrenamiento-en-patinodromo/</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Cinco hombres fueron asesinados en Mocoa. El hecho se dio después de que se difundió un panfleto amenazante.</t>
+          <t>El joven hacía parte de la Liga Vallecaucana de Patinaje y del club Relámpago.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Patinador de 14 años de la Liga Vallecaucana murió durante un entrenamiento: esto se sabe</t>
+          <t>Capturan a hombre que se hizo pasar por mototaxista y abusó de una joven de 14 años en Cali</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Popayán</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -7866,34 +7866,34 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/muere-joven-patinador-en-cali-tras-accidente-durante-entrenamiento-en-patinodromo/</t>
+          <t>https://www.elespectador.com/colombia/cali/capturan-a-hombre-que-se-hizo-pasar-por-mototaxista-y-abuso-de-una-joven-de-14-anos-en-cali/</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>El joven hacía parte de la Liga Vallecaucana de Patinaje y del club Relámpago.</t>
+          <t>La víctima fue herida con arma cortopunzante y asfixiada hasta quedar inconsciente.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Capturan a hombre que se hizo pasar por mototaxista y abusó de una joven de 14 años en Cali</t>
+          <t>La jueza que investiga el colapso de una pasarela en Santander imputa a un tercer técnico de Costas y aprecia indicios de seis homicidios por imprudencia grave</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bucaramanga</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -7913,12 +7913,12 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/capturan-a-hombre-que-se-hizo-pasar-por-mototaxista-y-abuso-de-una-joven-de-14-anos-en-cali/</t>
+          <t>https://www.infobae.com/espana/2026/04/21/la-jueza-que-investiga-el-colapso-de-una-pasarela-en-santander-imputa-a-un-tercer-tecnico-de-costas-y-aprecia-indicios-de-seis-homicidios-por-imprudencia-grave/</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>La víctima fue herida con arma cortopunzante y asfixiada hasta quedar inconsciente.</t>
+          <t>La instructora considera que la falta de inspección y mantenimiento durante años generó un riesgo no controlado que desembocó en el desplome de la estructura y en la muerte de seis jóvenes</t>
         </is>
       </c>
     </row>
@@ -7930,17 +7930,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>La jueza que investiga el colapso de una pasarela en Santander imputa a un tercer técnico de Costas y aprecia indicios de seis homicidios por imprudencia grave</t>
+          <t>Investigan el asesinato de adolescente de 15 años en campo de golf en Cartagena</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Bucaramanga</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -7960,34 +7960,34 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/espana/2026/04/21/la-jueza-que-investiga-el-colapso-de-una-pasarela-en-santander-imputa-a-un-tercer-tecnico-de-costas-y-aprecia-indicios-de-seis-homicidios-por-imprudencia-grave/</t>
+          <t>https://www.elespectador.com/colombia/cartagena/investigan-el-asesinato-de-adolescente-de-17-anos-en-campo-de-golf-en-cartagena/</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>La instructora considera que la falta de inspección y mantenimiento durante años generó un riesgo no controlado que desembocó en el desplome de la estructura y en la muerte de seis jóvenes</t>
+          <t>Las autoridades buscan esclarecer por qué un empleado de seguridad de un club de golf de Cartagena disparó contra un adolescente.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Investigan el asesinato de adolescente de 15 años en campo de golf en Cartagena</t>
+          <t>Filtran las primeras imágenes del doble asesinato contra miembros de la producción de ‘Sin senos sí hay paraíso 4′ en Bogotá: el agresor atacó por la espalda</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -7997,34 +7997,34 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cartagena/investigan-el-asesinato-de-adolescente-de-17-anos-en-campo-de-golf-en-cartagena/</t>
+          <t>https://www.infobae.com/colombia/2026/04/20/filtran-las-primeras-imagenes-del-doble-asesinato-contra-miembros-de-la-produccion-de-sin-senos-si-hay-paraiso-4-en-bogota-el-agresor-ataco-por-la-espalda/</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Las autoridades buscan esclarecer por qué un empleado de seguridad de un club de golf de Cartagena disparó contra un adolescente.</t>
+          <t>En el material fílmico se observa cuando el joven de 24 años diagnosticado con enfermedad mental se acercó al conductor de 45 años y, sin mediar palabra, lo tomó por el cuello y lo hirió mortalmente con arma blanca</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Filtran las primeras imágenes del doble asesinato contra miembros de la producción de ‘Sin senos sí hay paraíso 4′ en Bogotá: el agresor atacó por la espalda</t>
+          <t>Magnicidio Miguel Uribe Turbay: menor de edad que disparó al precandidato fue declarado como víctima en el proceso judicial</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -8044,39 +8044,39 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/04/20/filtran-las-primeras-imagenes-del-doble-asesinato-contra-miembros-de-la-produccion-de-sin-senos-si-hay-paraiso-4-en-bogota-el-agresor-ataco-por-la-espalda/</t>
+          <t>https://www.infobae.com/colombia/2026/04/18/magnicidio-miguel-uribe-turbay-menor-de-edad-que-disparo-al-precandidato-fue-declarado-como-victima-en-el-proceso-judicial/</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>En el material fílmico se observa cuando el joven de 24 años diagnosticado con enfermedad mental se acercó al conductor de 45 años y, sin mediar palabra, lo tomó por el cuello y lo hirió mortalmente con arma blanca</t>
+          <t>Alias Tianz confesó el crimen y cumple una sanción de siete años en un centro de atención especializada, bajo la custodia del Instituto Colombiano de Bienestar Familiar</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Magnicidio Miguel Uribe Turbay: menor de edad que disparó al precandidato fue declarado como víctima en el proceso judicial</t>
+          <t>Uno de cada cuatro jovenes en colombia no estudia ni trabaja y el mercado laboral da senales de debilidad</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Portafolio</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -8101,14 +8101,10 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/04/18/magnicidio-miguel-uribe-turbay-menor-de-edad-que-disparo-al-precandidato-fue-declarado-como-victima-en-el-proceso-judicial/</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>Alias Tianz confesó el crimen y cumple una sanción de siete años en un centro de atención especializada, bajo la custodia del Instituto Colombiano de Bienestar Familiar</t>
-        </is>
-      </c>
+          <t>https://www.portafolio.co/economia/empleo/uno-de-cada-cuatro-jovenes-en-colombia-no-estudia-ni-trabaja-y-el-mercado-laboral-da-senales-de-debilidad-492018</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8118,60 +8114,64 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Uno de cada cuatro jovenes en colombia no estudia ni trabaja y el mercado laboral da senales de debilidad</t>
+          <t>¡Atención, jóvenes! Bogotá abre formación gratuita para impulsar emprendimientos</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Portafolio</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>https://www.portafolio.co/economia/empleo/uno-de-cada-cuatro-jovenes-en-colombia-no-estudia-ni-trabaja-y-el-mercado-laboral-da-senales-de-debilidad-492018</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ee67a6f4f1</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>•Bogotá abre la convocatoria de Innovers 2026, un programa gratuito para fortalecer el emprendimiento juvenil. • Dirigido a jóvenes entre 18 y 28 años, desde quienes tienen una idea hasta emprendimientos en crecimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>¡Atención, jóvenes! Bogotá abre formación gratuita para impulsar emprendimientos</t>
+          <t>Asesinaron a dos jóvenes que habían sido secuestrados por la guerrilla hace un mes en Arauca</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -8181,44 +8181,40 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Arauca</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ee67a6f4f1</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria de Innovers 2026, un programa gratuito para fortalecer el emprendimiento juvenil. • Dirigido a jóvenes entre 18 y 28 años, desde quienes tienen una idea hasta emprendimientos en crecimiento.</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/asesinaron-a-dos-jovenes-que-habian-sido-secuestrados-por-la-guerrilla-hace-un-mes-en-arauca-rg10</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Asesinaron a dos jóvenes que habían sido secuestrados por la guerrilla hace un mes en Arauca</t>
+          <t>Bomberos rescataron a joven que le quedó atrapado el dedo en una banca del MIO en Cali</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -8228,7 +8224,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Arauca</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -8238,20 +8234,24 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/asesinaron-a-dos-jovenes-que-habian-sido-secuestrados-por-la-guerrilla-hace-un-mes-en-arauca-rg10</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/bomberos-rescataron-a-joven-que-le-quedo-atrapado-el-dedo-en-una-banca-del-mio-en-cali/</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>El caso ocurrió en un paradero del sistema en el barrio Potrero Grande del MIO en Cali.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Bomberos rescataron a joven que le quedó atrapado el dedo en una banca del MIO en Cali</t>
+          <t>Medellín abre convocatoria para impulsar emprendimientos rurales de jóvenes y mujeres</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -8281,12 +8281,12 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/bomberos-rescataron-a-joven-que-le-quedo-atrapado-el-dedo-en-una-banca-del-mio-en-cali/</t>
+          <t>https://www.elespectador.com/colombia/medellin/medellin-abre-convocatoria-para-impulsar-emprendimientos-rurales-de-jovenes-y-mujeres/</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>El caso ocurrió en un paradero del sistema en el barrio Potrero Grande del MIO en Cali.</t>
+          <t>Hasta 40 iniciativas podrán acceder a recursos y acompañamiento técnico. Las inscripciones estarán abiertas hasta el 10 de abril.</t>
         </is>
       </c>
     </row>
@@ -8298,27 +8298,27 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Medellín abre convocatoria para impulsar emprendimientos rurales de jóvenes y mujeres</t>
+          <t>MATAR MUJERES: LA VIOLENCIA INSTRUMENTAL COMO ESTRATEGIA DEL CONTROL ARMADO</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -8328,34 +8328,34 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/medellin/medellin-abre-convocatoria-para-impulsar-emprendimientos-rurales-de-jovenes-y-mujeres/</t>
+          <t>https://www.lasillavacia.com/red-de-expertos/matar-mujeres-la-violencia-instrumental-como-estrategia-del-control-armado/</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Hasta 40 iniciativas podrán acceder a recursos y acompañamiento técnico. Las inscripciones estarán abiertas hasta el 10 de abril.</t>
+          <t>El asesinato de dos adolescentes en Malambo, Atlántico, es un crimen atroz que evidencia una lógica que se repite en distintos territorios y que consiste en matar mujeres para castigar, advertir e imponer control. Mientras sus familias recibían...</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>MATAR MUJERES: LA VIOLENCIA INSTRUMENTAL COMO ESTRATEGIA DEL CONTROL ARMADO</t>
+          <t>Capturan a joven de 19 años por asesinato de mujer y su hijo en Villavicencio</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Villavicencio</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -8375,12 +8375,12 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/red-de-expertos/matar-mujeres-la-violencia-instrumental-como-estrategia-del-control-armado/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/capturan-a-joven-de-19-anos-por-asesinato-de-mujer-y-su-hijo-en-villavicencio/</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>El asesinato de dos adolescentes en Malambo, Atlántico, es un crimen atroz que evidencia una lógica que se repite en distintos territorios y que consiste en matar mujeres para castigar, advertir e imponer control. Mientras sus familias recibían...</t>
+          <t>Las autoridades capturaron a un joven de 19 años señalado del doble homicidio ocurrido en el barrio San Antonio de Villavicencio.</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Capturan a joven de 19 años por asesinato de mujer y su hijo en Villavicencio</t>
+          <t>Hallaron el cuerpo de una adolescente de 14 años que se ahogó en playa de Antioquia</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -8407,12 +8407,12 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Villavicencio</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -8422,24 +8422,24 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/capturan-a-joven-de-19-anos-por-asesinato-de-mujer-y-su-hijo-en-villavicencio/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallaron-el-cuerpo-de-una-adolescente-de-14-anos-que-se-ahogo-en-playa-de-san-juan-de-uraba-en-antioquia/</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Las autoridades capturaron a un joven de 19 años señalado del doble homicidio ocurrido en el barrio San Antonio de Villavicencio.</t>
+          <t>La menor había ingresado al mar con una amiga en una zona con fuerte oleaje. Su cuerpo fue hallado horas después.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Hallaron el cuerpo de una adolescente de 14 años que se ahogó en playa de Antioquia</t>
+          <t>Ataque de pitbull que dejó a perro muerto y joven herido en Barranquilla</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -8454,12 +8454,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -8469,59 +8469,59 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallaron-el-cuerpo-de-una-adolescente-de-14-anos-que-se-ahogo-en-playa-de-san-juan-de-uraba-en-antioquia/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/anuncian-acciones-tras-ataque-de-pitbull-que-dejo-a-perro-muerto-y-joven-herido-en-barranquilla/</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>La menor había ingresado al mar con una amiga en una zona con fuerte oleaje. Su cuerpo fue hallado horas después.</t>
+          <t>El hecho ocurrió en un conjunto residencial de Barranquilla y quedó registrado en cámaras de seguridad.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Ataque de pitbull que dejó a perro muerto y joven herido en Barranquilla</t>
+          <t>Prosperidad Social amplía el periodo de transferencias de Renta Joven en modalidad de giro</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Política pública</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/barranquilla/anuncian-acciones-tras-ataque-de-pitbull-que-dejo-a-perro-muerto-y-joven-herido-en-barranquilla/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-amplia-el-periodo-de-transferencias-de-renta-joven-en-modalidad-de-giro/</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>El hecho ocurrió en un conjunto residencial de Barranquilla y quedó registrado en cámaras de seguridad.</t>
+          <t>La ampliación del plazo permitirá que más de 27.000 participantes reciban sus subsidios, incluyendo transferencias pendientes de 2025. La transferencia monetaria condicionada se podrá reclamar en los puntos autorizados de SuRed y SuperGIROS. Bogotá...</t>
         </is>
       </c>
     </row>
@@ -8533,12 +8533,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Prosperidad Social amplía el periodo de transferencias de Renta Joven en modalidad de giro</t>
+          <t>Nueva convocatoria dirigida a jóvenes interesados en formarse en el sector de gastronomía</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Política pública</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -8563,59 +8563,59 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-amplia-el-periodo-de-transferencias-de-renta-joven-en-modalidad-de-giro/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e5d592a6d5</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>La ampliación del plazo permitirá que más de 27.000 participantes reciban sus subsidios, incluyendo transferencias pendientes de 2025. La transferencia monetaria condicionada se podrá reclamar en los puntos autorizados de SuRed y SuperGIROS. Bogotá...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años, principalmente de la localidad de Kennedy, para formarse en servicio para el sector de la gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Nueva convocatoria dirigida a jóvenes interesados en formarse en el sector de gastronomía</t>
+          <t>La incoherente decisión de Petro de abrirle la Casa de Nariño a Westcol decepcionó a quienes respaldaban su gobierno</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e5d592a6d5</t>
+          <t>https://www.las2orillas.co/la-incoherente-decision-de-petro-de-abrirle-la-casa-de-narino-a-westcol-decepciono-a-quienes-respaldaban-su-gobierno/</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años, principalmente de la localidad de Kennedy, para formarse en servicio para el sector de la gastronomía. • Esta formación...</t>
+          <t>Recibir a Westcol tras la tragedia del Hércules y sus discursos de odio es un golpe a la coherencia progresista. ¿Vale todo por llegarle a los jóvenes?El artículoLa incoherente decisión de Petro de abrirle la Casa de Nariño a Westcol decepcionó a...</t>
         </is>
       </c>
     </row>
@@ -8627,12 +8627,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>La incoherente decisión de Petro de abrirle la Casa de Nariño a Westcol decepcionó a quienes respaldaban su gobierno</t>
+          <t>Primero Petro luego Uribe: Westcol, el streamer que entrevista presidentes</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -8657,12 +8657,12 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-incoherente-decision-de-petro-de-abrirle-la-casa-de-narino-a-westcol-decepciono-a-quienes-respaldaban-su-gobierno/</t>
+          <t>https://www.lasillavacia.com/silla-nacional/primero-petro-luego-uribe-westcol-el-streamer-que-entrevista-presidentes/</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Recibir a Westcol tras la tragedia del Hércules y sus discursos de odio es un golpe a la coherencia progresista. ¿Vale todo por llegarle a los jóvenes?El artículoLa incoherente decisión de Petro de abrirle la Casa de Nariño a Westcol decepcionó a...</t>
+          <t>El influencer se convierte en interlocutor de los dos políticos más poderosos de Colombia. Ambos van detrás de su audiencia joven y masiva en época electoral.The postPrimero Petro luego Uribe: Westcol, el streamer que entrevista presidentesappeared...</t>
         </is>
       </c>
     </row>
@@ -8674,27 +8674,27 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Primero Petro luego Uribe: Westcol, el streamer que entrevista presidentes</t>
+          <t>Asesinaron a joven futbolista en Barranquilla; le dispararon en la cabeza</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -8704,24 +8704,24 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/silla-nacional/primero-petro-luego-uribe-westcol-el-streamer-que-entrevista-presidentes/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/asesinaron-a-joven-futbolista-en-barranquilla-le-dispararon-en-la-cabeza/</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>El influencer se convierte en interlocutor de los dos políticos más poderosos de Colombia. Ambos van detrás de su audiencia joven y masiva en época electoral.The postPrimero Petro luego Uribe: Westcol, el streamer que entrevista presidentesappeared...</t>
+          <t>Asesinaron a una joven promesa del fútbol en el barrio El Santuario de Barranquilla. Le dispararon en la cabeza en medio de una riña.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Asesinaron a joven futbolista en Barranquilla; le dispararon en la cabeza</t>
+          <t>Asesinaron a dos jóvenes en ataque sicarial en una discoteca de Riohacha</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -8741,7 +8741,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Riohacha</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -8751,12 +8751,12 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/barranquilla/asesinaron-a-joven-futbolista-en-barranquilla-le-dispararon-en-la-cabeza/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/tres-sicarios-abrieron-fuego-en-una-discoteca-de-riohacha-y-asesinaron-dos-jovenes/</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Asesinaron a una joven promesa del fútbol en el barrio El Santuario de Barranquilla. Le dispararon en la cabeza en medio de una riña.</t>
+          <t>¿Qué sucedió en el ataque de tres sicarios ocurrido en una discoteca de Riohacha?</t>
         </is>
       </c>
     </row>
@@ -8768,69 +8768,69 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Asesinaron a dos jóvenes en ataque sicarial en una discoteca de Riohacha</t>
+          <t>Así fue la participación de los jóvenes en el primer Fest de las Oportunidades del año</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Riohacha</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/tres-sicarios-abrieron-fuego-en-una-discoteca-de-riohacha-y-asesinaron-dos-jovenes/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9690ed7762</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>¿Qué sucedió en el ataque de tres sicarios ocurrido en una discoteca de Riohacha?</t>
+          <t>•El primer Fest de las Oportunidades 2026 reunió a más de 130 jóvenes en Usme, conectándolos con oferta en empleo, educación, emprendimiento y bienestar. •Más de 20 entidades y aliados participaron acercando oportunidades reales y orientación...</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Así fue la participación de los jóvenes en el primer Fest de las Oportunidades del año</t>
+          <t>Conductor atropelló y mató a un joven en Bogotá tras invadir el carril exclusivo de Transmilenio</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -8845,12 +8845,12 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9690ed7762</t>
+          <t>https://www.infobae.com/colombia/2026/03/28/conductor-atropello-y-mato-a-un-joven-en-bogota-tras-invadir-el-carril-exclusivo-de-transmilenio/</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>•El primer Fest de las Oportunidades 2026 reunió a más de 130 jóvenes en Usme, conectándolos con oferta en empleo, educación, emprendimiento y bienestar. •Más de 20 entidades y aliados participaron acercando oportunidades reales y orientación...</t>
+          <t>La muerte de Juan Sebastián Triviño y las lesiones sufridas por su acompañante mantienen en alerta a la ciudad, mientras los familiares reclaman las grabaciones de cámaras de seguridad como elemento determinante para identificar al conductor...</t>
         </is>
       </c>
     </row>
@@ -8862,22 +8862,22 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Conductor atropelló y mató a un joven en Bogotá tras invadir el carril exclusivo de Transmilenio</t>
+          <t>Sobre la entrega de transferencias monetarias condicionadas de Jóvenes en Paz</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -8892,12 +8892,12 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/28/conductor-atropello-y-mato-a-un-joven-en-bogota-tras-invadir-el-carril-exclusivo-de-transmilenio/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/sobre-la-entrega-de-transferencias-monetarias-condicionadas-de-jovenes-en-paz/</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>La muerte de Juan Sebastián Triviño y las lesiones sufridas por su acompañante mantienen en alerta a la ciudad, mientras los familiares reclaman las grabaciones de cámaras de seguridad como elemento determinante para identificar al conductor...</t>
+          <t>Bogotá D.C., 27 de marzo de 2026. Prosperidad Social informa a los participantes del programa Jóvenes en Paz que se adelanta la última etapa del procedimiento para disponer de los recursos de los próximos ciclos del año. En consecuencia: La entrega...</t>
         </is>
       </c>
     </row>
@@ -8909,54 +8909,54 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Sobre la entrega de transferencias monetarias condicionadas de Jóvenes en Paz</t>
+          <t>Continúa la búsqueda de cuatro jóvenes desaparecidos en Coromoro, Santander</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/sobre-la-entrega-de-transferencias-monetarias-condicionadas-de-jovenes-en-paz/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/buscan-a-cuatro-jovenes-desaparecidos-en-coromoro-santander-noticias-hoy/</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Bogotá D.C., 27 de marzo de 2026. Prosperidad Social informa a los participantes del programa Jóvenes en Paz que se adelanta la última etapa del procedimiento para disponer de los recursos de los próximos ciclos del año. En consecuencia: La entrega...</t>
+          <t>Inicialmente eran seis los reportados como desaparecidos.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Continúa la búsqueda de cuatro jóvenes desaparecidos en Coromoro, Santander</t>
+          <t>La historia de Luis Fernando Hostia y la meta de abrir caminos a personas con discapacidad</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -8986,24 +8986,24 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/buscan-a-cuatro-jovenes-desaparecidos-en-coromoro-santander-noticias-hoy/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/la-historia-de-luis-fernando-hostia-y-la-meta-de-romper-barreras-a-personas-con-discapacidad/</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Inicialmente eran seis los reportados como desaparecidos.</t>
+          <t>Desde San Sebastián de Buenavista, un joven en condición de discapacidad rompió décadas de barreras educativas.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>La historia de Luis Fernando Hostia y la meta de abrir caminos a personas con discapacidad</t>
+          <t>Lo que se sabe de la muerte de joven dentro de Univalle; hay varias preguntas</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -9018,12 +9018,12 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -9033,24 +9033,24 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/la-historia-de-luis-fernando-hostia-y-la-meta-de-romper-barreras-a-personas-con-discapacidad/</t>
+          <t>https://www.elespectador.com/colombia/cali/lo-que-se-sabe-de-la-muerte-de-joven-dentro-de-univalle-hay-varias-preguntas/</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Desde San Sebastián de Buenavista, un joven en condición de discapacidad rompió décadas de barreras educativas.</t>
+          <t>El caso ocurrió durante el fin de semana en la sede Meléndez de la Universidad del Valle, en Cali. La Secretaría de Movilidad se pronunció.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Lo que se sabe de la muerte de joven dentro de Univalle; hay varias preguntas</t>
+          <t>Buscan a joven que desapareció en río Lebrija en Santander en medio de fuertes lluvias</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -9065,12 +9065,12 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -9080,24 +9080,24 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/lo-que-se-sabe-de-la-muerte-de-joven-dentro-de-univalle-hay-varias-preguntas/</t>
+          <t>https://www.elespectador.com/colombia/buscan-a-joven-que-desaparecio-en-rio-lebrija-en-santander-en-medio-de-fuertes-lluvias/</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>El caso ocurrió durante el fin de semana en la sede Meléndez de la Universidad del Valle, en Cali. La Secretaría de Movilidad se pronunció.</t>
+          <t>Un joven de 24 años desapareció en el río Lebrija tras ser arrastrado por corriente. Las lluvias dejan más de 140 familias damnificadas.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Buscan a joven que desapareció en río Lebrija en Santander en medio de fuertes lluvias</t>
+          <t>Balacera en Barranquilla dejó tres personas heridas y tres capturadas</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -9112,12 +9112,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -9127,71 +9127,67 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/buscan-a-joven-que-desaparecio-en-rio-lebrija-en-santander-en-medio-de-fuertes-lluvias/</t>
+          <t>https://www.elespectador.com/colombia/barranquilla/balacera-en-barranquilla-dejo-tres-personas-heridas-y-tres-capturadas/</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Un joven de 24 años desapareció en el río Lebrija tras ser arrastrado por corriente. Las lluvias dejan más de 140 familias damnificadas.</t>
+          <t>Una balacera, al parecer entre miembros de Pepes y Costeños, dejó tres heridos y tres capturados, entre ellos un menor de edad.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Balacera en Barranquilla dejó tres personas heridas y tres capturadas</t>
+          <t>Insólito pedido de familia de David Acosta luego de que el joven apareciera con vida en Bogotá</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/barranquilla/balacera-en-barranquilla-dejo-tres-personas-heridas-y-tres-capturadas/</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>Una balacera, al parecer entre miembros de Pepes y Costeños, dejó tres heridos y tres capturados, entre ellos un menor de edad.</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/caso-david-acosta-familia-pide-cerrar-investigacion-falsa-desaparicion-PP5103111</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Insólito pedido de familia de David Acosta luego de que el joven apareciera con vida en Bogotá</t>
+          <t>Colombia tendrá más viejos que jóvenes a partir de esta fecha; hay alerta por las pensiones</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -9211,17 +9207,17 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/caso-david-acosta-familia-pide-cerrar-investigacion-falsa-desaparicion-PP5103111</t>
+          <t>https://www.pulzo.com/economia/colombia-tendra-mas-viejos-que-jovenes-partir-esta-fecha-hay-alerta-PP5100998A</t>
         </is>
       </c>
       <c r="I190" t="inlineStr"/>
@@ -9234,27 +9230,27 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Colombia tendrá más viejos que jóvenes a partir de esta fecha; hay alerta por las pensiones</t>
+          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -9264,30 +9260,34 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/economia/colombia-tendra-mas-viejos-que-jovenes-partir-esta-fecha-hay-alerta-PP5100998A</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr"/>
+          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Adolescente de 14 años murió en riña entre menores de edad fuera de un colegio en Cali</t>
+          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -9297,81 +9297,81 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/adolescente-de-14-anos-murio-en-rina-entre-menores-de-edad-fuera-de-un-colegio-en-cali/</t>
+          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Adolescente de 14 años murió en riña entre menores afuera de un colegio en Cali. ¿Qué dicen las autoridades?</t>
+          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Mafe Carrascal explicó por qué la bancada del Pacto Histórico por Bogotá no asistió a encuentro con el alcalde Carlos Fernando Galán</t>
+          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/17/mafe-carrascal-explico-por-que-la-bancada-del-pacto-historico-por-bogota-no-asistio-a-encuentro-con-el-alcalde-carlos-fernando-galan/</t>
+          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>La representante indicó que la reunión se realizaría a puerta cerrada y que esta decisión contradice los intereses de su partido. Además, afirmó que al gobierno local le falta implementar políticas dirigidas a los jóvenes y a la prevención de...</t>
+          <t>El presunto homicida ya fue localizado y detenido.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Asesinan a joven de 15 años en Cartagena; su padre resultó herido al intentar defenderlo</t>
+          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -9386,12 +9386,12 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -9401,12 +9401,12 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/asesinan-a-menor-de-15-anos-en-cartagena-su-padre-resulto-herido-al-intentar-defenderlo/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>El presunto homicida ya fue localizado y detenido.</t>
+          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
         </is>
       </c>
     </row>
@@ -9418,7 +9418,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Hallan el cuerpo de una adolescente en vivienda de Sahagún, Córdoba; autoridades investigan</t>
+          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -9448,44 +9448,44 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/hallan-el-cuerpo-de-una-menor-en-una-vivienda-de-sahagun-cordoba-autoridades-investigan/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>En lo que va de este año, este sería el tercer caso de una mujer asesinada en el municipio y el cuarto en el departamento.</t>
+          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Dos jóvenes fueron detenidos por presunta extorsión en Santo Tomás, Atlántico</t>
+          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -9495,29 +9495,29 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-jovenes-fueron-detenidos-por-presunta-extorsion-en-santo-tomas-atlantico/</t>
+          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>La investigación señala que los implicados habrían intimidado a un conductor de furgón.</t>
+          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Con $86 mil millones de regalías, Bolívar construirá universidad en Montes de María y otros dos proyectos educativos</t>
+          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -9527,12 +9527,12 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -9542,57 +9542,57 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-86-mil-millones-de-regalias-bolivar-construira-universidad-en-montes-de-maria-y-otros-dos-proyectos-educativos/</t>
-        </is>
-      </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>Los proyectos impulsados por Yamil Arana buscan, entre otras cosas, abrir más de 4 mil cupos para jóvenes de una región que durante años fue escenario de conflictoEl artículoCon $86 mil millones de regalías, Bolívar construirá universidad en Montes...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Nuevo giro en el caso de Tatiana Hernández, joven desaparecida en Cartagena: la buscan en el mar</t>
+          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/caso-tatiana-hernandez-da-giro-autoridades-intensifican-busqueda-mar-PP5091130</t>
-        </is>
-      </c>
-      <c r="I198" t="inlineStr"/>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Prosperidad Social responde a inquietudes sobre Renta Joven</t>
+          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -9632,12 +9632,12 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-responde-a-inquietudes-sobre-renta-joven/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Bogotá D. C, 4 de marzo de 2026. Prosperidad Social se permite aclarar a la ciudadanía y, especialmente, a los participantes de Renta Joven algunas dudas e inquietudes que han expresado los beneficiarios en las redes sociales. Prosperidad Social...</t>
+          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
         </is>
       </c>
     </row>
@@ -9649,42 +9649,42 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Maratón por las generaciones atendió a más de 38.000 jóvenes y personas mayores beneficiarias de Prosperidad Social</t>
+          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/maraton-por-las-generaciones-atendio-a-mas-de-38-000-jovenes-y-personas-mayores-beneficiarias-de-prosperidad-social/</t>
+          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Durante 38 horas continuas, se resolvieron inquietudes y dudas a beneficiarias y beneficiarios de los programas Renta Joven y Colombia Mayor. Nueve de cada 10 personas afirmaron haber recibido información clara y efectiva para resolver sus...</t>
+          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
         </is>
       </c>
     </row>
@@ -9696,42 +9696,42 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Joven rompió el silencio y reveló desgarradores detalles de los feminicidios más brutales del Valle del Cauca</t>
+          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/joven-rompio-el-silencio-y-revelo-desgarradores-detalles-de-los-feminicidios-mas-brutales-del-valle-del-cauca/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Mientras la Fiscalía la señala de disparar contra las víctimas, Angy Pérez asegura que fue obligada a desmembrar los cuerpos bajo la amenaza de perder a su bebéEl artículoJoven rompió el silencio y reveló desgarradores detalles de los feminicidios...</t>
+          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
         </is>
       </c>
     </row>
@@ -9743,101 +9743,101 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Colombia Mayor y Renta Joven: Prosperidad Social realizará la Maratón por las Generaciones</t>
+          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/colombia-mayor-y-renta-joven-prosperidad-social-realizara-la-maraton-por-las-generaciones/</t>
+          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Se trata de una jornada continua de atención telefónica, en la que se resolverán inquietudes que tengan beneficiarias y beneficiarios de estos dos programas de la entidad. El canal telefónico tendrá atención continua por más de 36 horas, mientras...</t>
+          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Así fue la despedida de Iván Zuleta a su sobrina Daniela: la joven fue encontrada sin signos vitales en su habitación</t>
+          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/03/11/asi-fue-la-despedida-de-ivan-zuleta-a-su-sobrina-daniela-que-habria-sido-encontrada-sin-signos-vitales-en-su-habitacion/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>La partida de la joven Zuleta Gnecco, hija de Fabián Zuleta y nieta de Fabio Zuleta, ha conmovido al mundo del vallenato, reuniendo a familiares y músicos icónicos para despedirla en Valledupar con emotivas muestras de cariño</t>
+          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Jóvenes en San Cristóbal inician su formación en servicio para el sector de la gastronomía</t>
+          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -9867,24 +9867,24 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#79ade27adc</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>•24 chicos y chicas iniciaron su camino en la Academia Ñam, en donde se formarán en servicio a la mesa para mejorar sus oportunidades de empleabilidad en el sector de la gastronomía. •La inducción, que tuvo lugar en el Centro de Desarrollo...</t>
+          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Bogotá presenta estudio que analiza los factores asociados a la vinculación de adolescentes a conductas punibles</t>
+          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -9899,7 +9899,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
@@ -9914,34 +9914,34 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#fb504c6e8d</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>• La vinculación de adolescentes a conductas punibles no responde a una sola causa, sino a la convergencia de factores estructurales, familiares, territoriales y personales que requieren respuestas integrales y no únicamente punitivas. • El consumo...</t>
+          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>La Academia Ñam llega a San Cristóbal con oportunidades para los jóvenes interesados en el sector de la gastronomía</t>
+          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -9961,86 +9961,86 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#1e64cd90aa</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>•El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio para el sector de la gastronomía. •Esta formación gratuita ofrece capacitación a...</t>
+          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>El deporte abrió la puerta a nuevas oportunidades y conexión para los jóvenes de Bogotá</t>
+          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>diario pago</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8b36ede0c2</t>
+          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>• En la localidad de Kennedy se realizó una jornada deportiva con Futsala Colombia, que acercó a los jóvenes la oferta integral de servicios sociales, digitales y educativos en territorio. • En Jóvenes con Oportunidades, más de 18.000 jóvenes han...</t>
+          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Abre 320 becas a jóvenes con proyectos en sus comunidades o entornos, ¿cómo participar?</t>
+          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
@@ -10055,24 +10055,24 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/abre-320-becas-a-jovenes-con-proyectos-en-sus-comunidades-o-entornos-como-participar/</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Abren becas para jóvenes en Medellín, Santa Marta, Cartagena y Bogotá. Tendrán formación, mentorías y acceso a redes de liderazgo.</t>
+          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>La primera guardia afro urbana liderada por mujeres surge en Cali</t>
+          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -10087,12 +10087,12 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -10102,24 +10102,24 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/cali/la-primera-guardia-afro-urbana-liderada-por-mujeres-surge-en-cali/</t>
+          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>En Llano Verde, mujeres desplazadas crearon la primera guardia afro urbana del país para prevenir violencia y proteger a jóvenes.</t>
+          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Bogotá fortalece el proceso de preinscripción de Jóvenes con Oportunidades 2026 y habilita nuevo enlace</t>
+          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -10149,81 +10149,77 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#6c31bba0c9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>•El Distrito habilitó un nuevo enlace mejorado para garantizar una experiencia más ágil, estable y segura en la convocatoria 2026 de Jóvenes con Oportunidades. •Las y los jóvenes entre 14 y 28 años que vivan en Bogotá y estén clasificados en Sisbén...</t>
+          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Aumenta el número de desaparecidos en Córdoba, dos jóvenes arrastrados por un arroyo</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>diario pago</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/colombia/mas-regiones/dos-campesinos-en-cordoba-desaparecen-tras-intentar-cruzar-un-arroyo/</t>
-        </is>
-      </c>
-      <c r="I211" t="inlineStr">
-        <is>
-          <t>Dos jóvenes campesinos permanecen desaparecidos en Córdoba, luego de que una corriente los arrastrara en cuanto intentaban cruzar un arroyo</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Bogotá abre convocatoria 2026 del programa Jóvenes con Oportunidades con más de 12.000 nuevos cupos</t>
+          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -10243,24 +10239,20 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#9a0f0687f3</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr">
-        <is>
-          <t>• El Distrito abre estaconvocatoria de Jóvenes con Oportunidades con más de 8.000 nuevos cupos, en su primera etapa, para jóvenes entre 14 y 28 años de Bogotá, fortaleciendo su acceso a rutas de formación, acompañamiento psicosocial y transferencias...</t>
-        </is>
-      </c>
+          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -10275,22 +10267,22 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdg?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
         </is>
       </c>
       <c r="I213" t="inlineStr"/>
@@ -10298,27 +10290,27 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Menores de edad mataron de 17 puñaladas a un hombre que iba de polizón en un camión de carga en la vía Bogotá-Villavicencio: quedó en video - Infobae</t>
+          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -10333,20 +10325,24 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxNYWQxNTA1UWhDOUtWS2dSWXNNQ19idDVRNXV4aktnZzFERmdBaFg0c2lrT2plR0tXcDN1dlFhd0J0Q1BUVmJEVU1YYTR3N0NtQUx2LTQ3amhNR2pNc0tvcjR6X1FfbkIwczFROFJTaFotclVpRGxId2h1eWtqbHMzSkNXc0JCeU1DWjkxOG5qekx4YjZGRlVVckdyX1gyT0luR2Nkd3ZQUTNFM1d1LUlvMzNSSGxiQUZ5V2pqT2E4WXhZWWRpY2JheDhpaWhwOTQwLThDWFlXU1p0N0lZVk5nSHdVZU8zWVlKNE9GTVJKaUxYTkxDMUt1MTF0NzN5MVUxXzBNUjZtZVJsWm9zMkNNdtIBqwJBVV95cUxPZnpNT2FPSmdUeFl0UmFScGh6MzVlYm9tVWhQekJjVTdRcHM2ZDlEbWFhVUJBX3dudVF2V01OaDdSRWN6c1FXV2thM0VJOHppRWhaWEVpbTVPOTVTd3RKcmJLT1NHa2MwVlR5SzE2TzlHM0RLS3k2VzFKRDdtaTd2M3RCNENTeXByY1BBTjR1SFE3STJQS3JBWURBRER1cTBKQmx2MVR6Sk5xYlpwbTdpNGRyWVBYdmkxTU9JaWNtRlZVM2JzTGtMQUhxaHFnUmVPQlNPbkNYWGlBX2ttc0Y4cjVzR0dVaFBER3lSMWxRZGVGVTRhTFZ6RE82ZzFKeWJnQ0U0bWlINmlXRE9KdUJvbzdpSEg1NURXMzZKeVNHWTd4b0puVldnbFlscw?oc=5</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Jóvenes narraron el calvario sufrido cuando fueron víctimas de presunto abuso en la Universidad de Cartagena: “Causó un gran sangrado”</t>
+          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -10361,22 +10357,22 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/02/02/jovenes-narraron-el-calvario-sufrido-cuando-fueron-victimas-de-presunto-abuso-en-la-universidad-de-cartagena-causo-un-gran-sangrado/</t>
+          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
         </is>
       </c>
       <c r="I215" t="inlineStr"/>
@@ -10384,74 +10380,70 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Bogotá abre nueva convocatoria de Academia Ñam para fortalecer la empleabilidad juvenil en el sector gastronómico</t>
+          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Sin identificar</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#85a520b8bc</t>
-        </is>
-      </c>
-      <c r="I216" t="inlineStr">
-        <is>
-          <t>• La Secretaría Distrital de Integración Social, en alianza con la Fundación Gastronomía Social, abre una nueva convocatoria de Academia Ñam, un programa gratuito de formación y práctica laboral en servicio gastronómico dirigido a jóvenes de 18 a 30...</t>
-        </is>
-      </c>
+          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Frustraron robo en un restaurante en Bosa, Bogotá: un hombre de 23 años y dos menores de edad fueron capturados</t>
+          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
@@ -10466,25 +10458,29 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/27/frustraron-robo-en-un-restaurante-en-bosa-bogota-un-hombre-de-23-anos-y-dos-menores-de-edad-fueron-capturados/</t>
-        </is>
-      </c>
-      <c r="I217" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Alerta en Tolima: ya son 4 los muertos por fiebre amarilla en 2026, entre ellos un menor de edad</t>
+          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -10494,12 +10490,12 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Sin identificar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -10509,7 +10505,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/alerta-en-tolima-ya-son-4-los-muertos-por-fiebre-amarilla-en-2026-entre-ellos-un-menor-de-edad-rg10</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
         </is>
       </c>
       <c r="I218" t="inlineStr"/>
@@ -10522,7 +10518,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Distrito Joven acompañó a más de 50 mil jóvenes en la construcción de sus proyectos de vida durante 2025</t>
+          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -10537,7 +10533,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -10552,24 +10548,24 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#729a4b8e04</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>• Durante 2025, la Subdirección para la Juventud acompañó a más de 50 mil jóvenes en Bogotá, fortaleciendo sus proyectos de vida a través de una atención integral. • Los servicios y estrategias implementados promovieron la inclusión social,...</t>
+          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Radiografía de los ‘ninis’ en Colombia: 2,26 millones de jóvenes están desconectados del estudio y el empleo - Infobae</t>
+          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -10584,7 +10580,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -10599,7 +10595,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQQzU0U2tHY3lvTUVKRmR2SExOeUdySS0ycnZSVWd3MlhIQmJmYVZxNm9NNVZ2YU8wZ1MtcUJiOXRPLWZhWUNLcUtVdG1uUVVUd0VfYU5sQWVNSjlDVWdDUTc2ZG8yajJIUlk0bVJxTTR3clhjd0wwRl9wSTRSUlk0UnZtY2FZTWZ2QUhQbjJ1TkdibEw4YmU4YXNTMEJUeV85V0dfSzdUQ0hSSk5DbFdZUk5VV2dnaGdabHhVQ1p2bjlCTlVKNHJNV3NoNmQtcG9CUkZaMWVDVXZmWDFXSTIxVi00UdIB_gFBVV95cUxQQXJkUXE5UnM4ZVhIZHo3UFJuSU0xVllueWt3Unk2aC03YllYdDBfc0FvalRGMDNsWjBRNmZfNUV1bTlsbWM3dFlLOGNCajVqcXQ5Z2hVRzdROXlpTUdrWEtLdVNyaDFqRGlnckQ3OUhfTjVNVk53YklESGhMMlRCcUVkNFRYMS04RUUwR2hvdERISVdENVlydzZhOGpfaU1yX0xkSkg0S3laV3E2MVV1UHRDN05aRU1iMlBiS2lRcXNWYTdMTlhVTzI2VkJkeFZTXzhqbS1adkpFa1RiX2dBaDJDaWhVYXVsM1psSV9jWjZGdy1QUXJ1d0xCdUxMdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
         </is>
       </c>
       <c r="I220" t="inlineStr"/>
@@ -10607,59 +10603,55 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Casas de Juventud lanzan nuevos Semilleros Distritales para potenciar el talento juvenil en Bogotá</t>
+          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>SDIS - Juventud</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#f8686f5026</t>
-        </is>
-      </c>
-      <c r="I221" t="inlineStr">
-        <is>
-          <t>•Bogotá abre la convocatoria a semilleros gratuitos en artes, deporte y cultura urbana, dirigidos a jóvenes entre 14 y 28 años de todas las localidades, como una estrategia distrital para fortalecer la expresión, la participación y el desarrollo de...</t>
-        </is>
-      </c>
+          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Estudio reveló las principales problemáticas que preocupan a los jóvenes en Colombia, previo a las elecciones de Congreso y Presidencia - Infobae</t>
+          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -10674,12 +10666,12 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -10689,7 +10681,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNYXdTSFVia3cwbnV6Y050TzB5M2JQckhpbDVVajdoRnZnZG1yTThKbVF0bFhsUWN0ZnFuM1h5M0VYWmxiUGZjaHN3WV85OFpwWlFaWkFkanlsSmcwNFhJQk5PTjJBZ3RXcTgzNHFCQU5qTGlUZlB3WTkxZmx3SVIwV05jblIwUFNNUUdBTkU2M2FZSHNlTUgyb2ZhZWsyMktyc0UtR2k2Z001NkUxZ01xSkxoei1uMUZqaGJfV0k2MWktaDVNRGtGOS1nNXlGTEdSZ1VSdEJGRDRkbkNPM3R1aURVbl9ZR3FYcC1aMkI4T0k4bDJaT0Jmb1dLNktqQVVOeHVpUGpkUGd3TmvSAaYCQVVfeXFMTl9Uc2p1OEVpYzZaLUFYOERNUjVQVjVSaHJtTEhhT1BibW1BMkVwQ0VVUFc3d2RsaWNtNHdTZm0tbDRlMHBPLWVES0Vyd3hKZHRQUmExYmVmaXNrZE5rTGhEWmd0YXQ5cjdPOGIyeVdEYUV5NHplUnFMX2pYWkRXdEFxbVB1UGhEOENhTWM3S2NCVnJQbDg4clVoSUhIWENVSUh1VE54MjZKUjF3OWdpUDZjdld4WU1BLTA2dWR2ZEwxQUpnLUNXS3JZZ2hWUkFQN2taQktacVNhM3NMOS1ZR1g2dkhmYmVmU0Q4Q0o2dWNCZUNMQnJsaDFjQlRXQUp5NUpEYllxWlhVQVVfbVlBdmVBa2RJRjVqNUNfTGxHMnFRaGhYMnN3?oc=5</t>
+          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
         </is>
       </c>
       <c r="I222" t="inlineStr"/>
@@ -10697,12 +10689,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Menor de edad colombiano fue baleado frente a su escuela en Chicago, la familia exige justicia</t>
+          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -10717,7 +10709,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -10732,7 +10724,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/14/menor-de-edad-colombiano-fue-baleado-frente-a-su-escuela-en-chicago-la-familia-exige-justicia/</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
         </is>
       </c>
       <c r="I223" t="inlineStr"/>
@@ -10740,12 +10732,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>El particular castigo de Policía en Barranquilla a un grupo de jóvenes quedó en video: “El cuerpo sufre”</t>
+          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -10760,12 +10752,12 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -10775,7 +10767,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/01/09/el-particular-castigo-de-policia-en-barranquilla-a-un-grupo-de-jovenes-quedo-en-video-el-cuerpo-sufre/</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
@@ -10783,98 +10775,106 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Aumenta a 1.419 el número de lesionados por pólvora en Colombia; 428 son menores de edad - Infobae</t>
+          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOY1FwS0xiWWVaYl9saTQ5X0xRYnVoR0lwNE5XYUVaaUl3LW8yN0hEZGFnckI5VVlrVnBPSFJpeDNkU1JIaC01dVJVdFJYbEtSVTFXRTBCdTFDSDJ6TXZjc2t5N0t0cVFUY2JGbGZ1NDB5R1FJVG1RX25hREVIMjZlYktrdHc2QUFiZXNQTXFGZk9zeWNJRUl1aWNCbG9OXzZRQVA2dFFUZ1J3UnJrZzU4Qnk5TVBMajBPenJOU0ZBekNheEl2SkV3QVRUc9IB5gFBVV95cUxQeDZfb0gzZm9CTTRpYWx1ZTBielQ1TVgtaHNBOXRVRjBDcVd2V3M2anR3VTJaLU8zUEFkbEJkdDFEcHdHQUlpNGVORDZXV1Jxdzl4YmdPN3F1bk10ODZ1MnpOUjVSRTZscUUzYl80MDVpaHROOXdBNlhoQkFFR3RyVVJ1MWw1WTVZZVcwWnZ6THBEYWkxR1hEMTQzRGIzRWJvWlVUOFFBU2duZE5MRnRoRnQyZDl0ajd2SEpUVVM5ZW5POEpzLUZIcTV1c3RaaHlvanRUcG1oU3REVFVVQk5xTnhuLWk1UQ?oc=5</t>
-        </is>
-      </c>
-      <c r="I225" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Gobierno condonará créditos del Icetex a más de mil jóvenes en Colombia: quiénes se beneficiarán - Infobae</t>
+          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>SDIS - Juventud</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Empleo</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOZlVSRmszbERPaGNNNjhFRXY3VGVlUjc0eXo5R002RDZTbk15NWlUb1pLeWtWdmtObV9fY2ZxUmQ3cHNacWJoMExhZVZDRjlJM0lYZ2VfUVJOTEJnOXhGeXhtOFdlX3BmdFZTWXNJWHpXSDJsREdSaXJHSmFfY0RCcV8xSFVTLThuS1M4eUwxYTMxdWU2WTY3YUVTaWtLWHJFRUhlM0EtQzFNdDQwNy1wU2NyMDIzSk5rZGI4ZExtcmx1b2R2d01DNzdZT29LanFzXzBaNjluZ0rSAfMBQVVfeXFMT3pmVy1QSHJLaTJmREJmLVNLano0XzdpeW1VemRocGF5eHBVZktPRnNkTnNBUElFMDk1UUQ4MTZRNENCVWpZQVhTRmNrV1dwbDhCQnFvemZKTmZyT2cwdV96a2xOUWZDZEloWEFKcjJ2QkJsX0h3bFZDTkNRNGJOY1U5UGZaN0x6YU1EQlN5ZlFLb0hYQkM1MDdKNWl5TS1OcVNYWHRGXzl5NFp1WnQ2YWJqcWZzZDlDTk5FQ19Sa2lZOXRpOEJ4LV9DUnVOenhkQ3FJUGhkZkExNkNOYlV2Z21iLUQxUmF0eDJ5c3NyekcxTFlF?oc=5</t>
-        </is>
-      </c>
-      <c r="I226" t="inlineStr"/>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Más de 40 jóvenes de Bogotá fueron reconocidos por su talento, creatividad y liderazgo en la Semana de la Juventud y la Semana Andina 2025</t>
+          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -10904,24 +10904,24 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c68de3a13a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>• Más de 40 jóvenes y colectivos fueron premiados por su creatividad, liderazgo y compromiso social durante la Semana de la Juventud y la Semana Andina 2025. • La Subdirección para la Juventud de la Secretaría Distrital de Integración Social abrió...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-10-09</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Jóvenes con Oportunidades abre convocatoria para su ruta de formación en cursos cortos</t>
+          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -10936,7 +10936,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Empleo</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -10951,24 +10951,24 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#28dd65106b</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>•La Subdirección para la Juventud anunció la apertura de nuevos cupos en la ruta de formación en cursos cortos, dirigida a jóvenes entre 18 y 28 años que vivan en Bogotá y cuenten con Sisbén IV (A1 a C09). • La ruta combina proyecto de vida, cursos...</t>
+          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>La Academia Ñam busca jóvenes interesados en el sector de la gastronomía</t>
+          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -10998,24 +10998,24 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#8622ae2557</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan una nueva convocatoria dirigida a jóvenes de 18 a 30 años de las localidades de La Candelaria y Santa Fe interesados en formarse en servicio en gastronomía. • Esta formación...</t>
+          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2025-10-09</t>
+          <t>2025-09-13</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>La Escuela Distrital de Emprendimiento ya está en marcha en Kennedy</t>
+          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -11045,24 +11045,24 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#09b7d9045f</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>• 50 jóvenes emprendedores fortalecerán sus proyectos de negocios de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento, que llega a su quinta edición, nace de la alianza del Distrito con la ANDI y la Fundación...</t>
+          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>La Academia Ñam abre una nueva convocatoria para jóvenes interesados en el sector de la gastronomía</t>
+          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -11092,24 +11092,24 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#17e48d890a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>• El Distrito, en alianza con la Fundación Gastronomía Social, lanzan convocatoria dirigida a jóvenes de 18 a 30 años interesados en formarse en servicio en el sector de la gastronomía. • Esta formación gratuita ofrece capacitación a través de...</t>
+          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>2025-09-13</t>
+          <t>2025-09-09</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Bogotá ofrece más de 1.500 becas para que jóvenes estudien programas técnicos laborales</t>
+          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -11139,24 +11139,24 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#e22c14d73a</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>•Se trata de la convocatoria Formación y Educación para el trabajo que les permitirá a los jóvenes de la ciudad formarse en una ocupación que requiere el mercado laboral. •Losbeneficiarios podrán estudiar mercadeo y ventas, mecánica dental, cocina,...</t>
+          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-09-06</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Jóvenes de la Casa de la Juventud de Suba aprenden sobre medio ambiente y navegan el río Bogotá</t>
+          <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -11186,104 +11186,10 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#ba7949b3a9</t>
+          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
-        <is>
-          <t>•Los navegantes confirmaron que los malos olores quedaron en el pasado y hoy se aprecian algunas especies de fauna que han comenzado a retornar a lo largo del cauce. • Gracias a la Corporación Autónoma Regional de Cundinamarca (CAR), encargada de...</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>2025-09-09</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>Está abierta la convocatoria para la Escuela Distrital de Emprendimiento en Kennedy</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>SDIS - Juventud</t>
-        </is>
-      </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Educación</t>
-        </is>
-      </c>
-      <c r="F234" t="inlineStr">
-        <is>
-          <t>Bogotá</t>
-        </is>
-      </c>
-      <c r="G234" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H234" t="inlineStr">
-        <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#2acaf10b23</t>
-        </is>
-      </c>
-      <c r="I234" t="inlineStr">
-        <is>
-          <t>• Jóvenes emprendedores podrán fortalecer sus proyectos de la mano de expertos y líderes empresariales. • La Escuela Distrital de Emprendimiento nace de la alianza del Distrito con la ANDI y la Fundación ANDI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>2025-09-06</t>
-        </is>
-      </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>El Frailejón abre sus puertas: Usme estrena nueva Casa de la Juventud</t>
-        </is>
-      </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>SDIS - Juventud</t>
-        </is>
-      </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>Otra</t>
-        </is>
-      </c>
-      <c r="F235" t="inlineStr">
-        <is>
-          <t>Bogotá</t>
-        </is>
-      </c>
-      <c r="G235" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H235" t="inlineStr">
-        <is>
-          <t>https://www.integracionsocial.gov.co/index.php/noticias/94-noticias-juventud#c7eca5d4bd</t>
-        </is>
-      </c>
-      <c r="I235" t="inlineStr">
         <is>
           <t>• Aunque ya existía una Casa de la Juventud en Usme, la sede se traslada y reinaugura para ofrecer mejores condiciones, ampliar servicios y fortalecer la atención a los jóvenes. • La reapertura se desarrolló con el acompañamiento de la Plataforma...</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-07
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>“La matan por ser mujer”: a diez años del crimen de Lucía Pérez, su madre insiste en que la Justicia lo califique como femicidio</t>
+          <t>La balcanización criminal de Haití</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -491,7 +491,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,59 +501,59 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/sociedad/policiales/2026/10/06/la-matan-por-ser-mujer-a-diez-anos-del-crimen-de-lucia-perez-su-madre-insiste-en-que-la-justicia-lo-califique-como-femicidio/</t>
+          <t>https://www.las2orillas.co/la-balcanizacion-criminal-de-haiti/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Marta Montero, la mamá de la joven asesinada en 2016 en Mar del Plata, atraviesa un nuevo aniversario del hecho mientras espera a que la Suprema Corte Bonaerense resuelva si el asesinato fue o no motivado por la cuestión de género</t>
+          <t>Puerto Príncipe su capital, es la ciudad más violenta del mundo. 200 pandillas ejercen una tenebrosa gobernanza criminalEl artículoLa balcanización criminal de Haitífue publicado originalmente enLas2orillas.co: Historias, voces y noticias de...</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>La balcanización criminal de Haití</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/la-balcanizacion-criminal-de-haiti/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Puerto Príncipe su capital, es la ciudad más violenta del mundo. 200 pandillas ejercen una tenebrosa gobernanza criminalEl artículoLa balcanización criminal de Haitífue publicado originalmente enLas2orillas.co: Historias, voces y noticias de...</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -565,42 +565,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>“La matan por ser mujer”: a diez años del crimen de Lucía Pérez, su madre insiste en que la Justicia lo califique como femicidio</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.infobae.com/sociedad/policiales/2026/10/06/la-matan-por-ser-mujer-a-diez-anos-del-crimen-de-lucia-perez-su-madre-insiste-en-que-la-justicia-lo-califique-como-femicidio/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>Marta Montero, la mamá de la joven asesinada en 2016 en Mar del Plata, atraviesa un nuevo aniversario del hecho mientras espera a que la Suprema Corte Bonaerense resuelva si el asesinato fue o no motivado por la cuestión de género</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-10
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,7 +466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -513,7 +513,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-12
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ocho clubes se consagran campeones en la Valledupar Cup 2026, que reunió a más de 3.500 jóvenes futbolistas</t>
+          <t>Gobierno anticipa anuncio sobre talento colombia: el plan para los jovenes que no estudian ni trabajan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Portafolio</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -491,7 +491,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Valledupar</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/deportes/futbol/valledupar-cup-2026-equipos-campeones-impacto-deportivo-y-economico-en-valledupar-colombia-PP5327651A</t>
+          <t>https://www.portafolio.co/economia/gobierno/gobierno-anticipa-anuncio-sobre-talento-colombia-el-plan-para-los-jovenes-que-no-estudian-ni-trabajan-504298</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -509,22 +509,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Polémica en Cúcuta por concejal que se peleó con un joven en un local comercial: “Vaya y mire quién soy yo”</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Infobae</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,22 +534,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cúcuta</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/10/11/polemica-en-cucuta-por-concejal-que-se-peleo-con-un-joven-en-un-local-comercial-vaya-y-mire-quien-soy-yo/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>La secuencia difundida en redes sociales muestra un intercambio verbal entre el cabildante Carlos Dueñas y un hombre al interior de un supermercado de la capital de Norte de Santander</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -561,12 +561,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sin el celular en los colegios, los jóvenes tendrán que enfrentarse a nueve horas de soledad</t>
+          <t>Ocho clubes se consagran campeones en la Valledupar Cup 2026, que reunió a más de 3.500 jóvenes futbolistas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -576,12 +576,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Educación</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Valledupar</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -591,14 +591,10 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/sin-el-celular-en-los-colegios-los-jovenes-tendran-que-enfrentarse-a-nueve-horas-de-soledad/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Limitar las pantallas en las escuelas es acertado, pero el debate de fondo es reconstruir los vínculos reales que hoy faltan en la adolescenciaEl artículoSin el celular en los colegios, los jóvenes tendrán que enfrentarse a nueve horas de soledadfue...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/deportes/futbol/valledupar-cup-2026-equipos-campeones-impacto-deportivo-y-economico-en-valledupar-colombia-PP5327651A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -608,17 +604,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Polémica en Cúcuta por concejal que se peleó con un joven en un local comercial: “Vaya y mire quién soy yo”</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Infobae</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -628,22 +624,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Cúcuta</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.infobae.com/colombia/2026/10/11/polemica-en-cucuta-por-concejal-que-se-peleo-con-un-joven-en-un-local-comercial-vaya-y-mire-quien-soy-yo/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>La secuencia difundida en redes sociales muestra un intercambio verbal entre el cabildante Carlos Dueñas y un hombre al interior de un supermercado de la capital de Norte de Santander</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-13
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,22 +466,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gobierno anticipa anuncio sobre talento colombia: el plan para los jovenes que no estudian ni trabajan</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Portafolio</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,20 +491,24 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.portafolio.co/economia/gobierno/gobierno-anticipa-anuncio-sobre-talento-colombia-el-plan-para-los-jovenes-que-no-estudian-ni-trabajan-504298</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,17 +518,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Gobierno anticipa anuncio sobre talento colombia: el plan para los jovenes que no estudian ni trabajan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Portafolio</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,24 +538,20 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
-        </is>
-      </c>
+          <t>https://www.portafolio.co/economia/gobierno/gobierno-anticipa-anuncio-sobre-talento-colombia-el-plan-para-los-jovenes-que-no-estudian-ni-trabajan-504298</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-19
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,22 +466,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Menor de edad rescatada tras quedar atrapada en accidente de tránsito en la variante Bogotá-Melgar, Cundinamarca</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -501,10 +501,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/accidente-en-variante-bogota-melgar-menor-atrapada-en-vehiculo-rescata-bomberos-en-melgar-cundinamarca-PP5333484A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,17 +518,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Menor de edad rescatada tras quedar atrapada en accidente de tránsito en la variante Bogotá-Melgar, Cundinamarca</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -544,14 +548,10 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/accidente-en-variante-bogota-melgar-menor-atrapada-en-vehiculo-rescata-bomberos-en-melgar-cundinamarca-PP5333484A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-22
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,12 +466,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>¿Por qué los colombianos caemos siempre en los mismos errores políticos?</t>
+          <t>Con 110 participantes en el Capitolio Nacional, el Congreso Juvenil pide espacio en la escena política</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -501,59 +501,59 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/por-que-los-colombianos-caemos-siempre-en-los-mismos-errores-politicos/</t>
+          <t>https://www.las2orillas.co/con-110-participantes-en-el-capitolio-nacional-el-congreso-juvenil-pide-espacio-en-la-escena-politica/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Una llamada a los jóvenes a conocer la historia política colombiana para evitar repetir errores del pasado y votar con verdadero sentido críticoEl artículo¿Por qué los colombianos caemos siempre en los mismos errores políticos?fue publicado...</t>
+          <t>Jóvenes colombianos simularon el ejercicio parlamentario en el Capitolio y abren el debate sobre las curules especiales para las nuevas generacionesEl artículoCon 110 participantes en el Capitolio Nacional, el Congreso Juvenil pide espacio en la...</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Por qué la llamada de su mamá que tardó 21 años en recibir salvó al humorista Iván Marín del suicidio</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/por-que-la-llamada-de-su-mama-que-tardo-21-anos-en-recibir-salvo-al-humorista-ivan-marin-del-suicidio/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>En el pódcast ‘La Habitación Invisible’, el comediante recordó la crisis existencial de la juventud y su recuperación en la que la comedia es protagonistaEl artículoPor qué la llamada de su mamá que tardó 21 años en recibir salvó al humorista Iván...</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -565,17 +565,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>¿Por qué los colombianos caemos siempre en los mismos errores políticos?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -585,22 +585,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.las2orillas.co/por-que-los-colombianos-caemos-siempre-en-los-mismos-errores-politicos/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>Una llamada a los jóvenes a conocer la historia política colombiana para evitar repetir errores del pasado y votar con verdadero sentido críticoEl artículo¿Por qué los colombianos caemos siempre en los mismos errores políticos?fue publicado...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-23
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,22 +466,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Con 110 participantes en el Capitolio Nacional, el Congreso Juvenil pide espacio en la escena política</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,22 +491,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/con-110-participantes-en-el-capitolio-nacional-el-congreso-juvenil-pide-espacio-en-la-escena-politica/</t>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Jóvenes colombianos simularon el ejercicio parlamentario en el Capitolio y abren el debate sobre las curules especiales para las nuevas generacionesEl artículoCon 110 participantes en el Capitolio Nacional, el Congreso Juvenil pide espacio en la...</t>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
         </is>
       </c>
     </row>
@@ -518,17 +518,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>Con 110 participantes en el Capitolio Nacional, el Congreso Juvenil pide espacio en la escena política</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -538,22 +538,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.las2orillas.co/con-110-participantes-en-el-capitolio-nacional-el-congreso-juvenil-pide-espacio-en-la-escena-politica/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>Jóvenes colombianos simularon el ejercicio parlamentario en el Capitolio y abren el debate sobre las curules especiales para las nuevas generacionesEl artículoCon 110 participantes en el Capitolio Nacional, el Congreso Juvenil pide espacio en la...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática de noticias - 2026-10-31
</commit_message>
<xml_diff>
--- a/data/noticias.xlsx
+++ b/data/noticias.xlsx
@@ -466,27 +466,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Festival de Libros para Niños y Jóvenes celebra su edición 20 en La Milla Encantada del Bronx Distrito Creativo en Bogotá</t>
+          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pulzo</t>
+          <t>Prosperidad Social</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>gratuito</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cultura y deporte</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -501,10 +501,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.pulzo.com/nacion/bogota/festival-de-libros-para-ninos-y-jovenes-2026-en-bogota-actividades-fecha-y-lugar-PP5345083A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,12 +518,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Guapi: donde navegar se convierte en liderazgo juvenil para transformar el Pacífico colombiano</t>
+          <t>Festival de Libros para Niños y Jóvenes celebra su edición 20 en La Milla Encantada del Bronx Distrito Creativo en Bogotá</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Las2orillas</t>
+          <t>Pulzo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -529,29 +533,25 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Cultura y deporte</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cali</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/guapi-donde-navegar-se-convierte-en-liderazgo-juvenil-para-transformar-el-pacifico-colombiano/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Desde Guapi hasta Cali, Angie Vanessa Montaño demuestra que la distancia geográfica y el abandono estatal no pueden seguir frenando a la juventud afroEl artículoGuapi: donde navegar se convierte en liderazgo juvenil para transformar el Pacífico...</t>
-        </is>
-      </c>
+          <t>https://www.pulzo.com/nacion/bogota/festival-de-libros-para-ninos-y-jovenes-2026-en-bogota-actividades-fecha-y-lugar-PP5345083A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>De huir del conflicto a llevar agua segura y sostenible a las aulas: el liderazgo de Mabel Garcés en el Cauca</t>
+          <t>Guapi: donde navegar se convierte en liderazgo juvenil para transformar el Pacífico colombiano</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -576,12 +576,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Violencia</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Popayán</t>
+          <t>Cali</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -591,12 +591,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.las2orillas.co/de-huir-del-conflicto-a-llevar-agua-segura-y-sostenible-a-las-aulas-el-liderazgo-de-mabel-garces-en-el-cauca/</t>
+          <t>https://www.las2orillas.co/guapi-donde-navegar-se-convierte-en-liderazgo-juvenil-para-transformar-el-pacifico-colombiano/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Desplazada en su niñez por la violencia, esta joven llevó a un colegio de Puerto Tejada un sistema de agua limpia pensado y cuidado por la propia comunidaEl artículoDe huir del conflicto a llevar agua segura y sostenible a las aulas: el liderazgo de...</t>
+          <t>Desde Guapi hasta Cali, Angie Vanessa Montaño demuestra que la distancia geográfica y el abandono estatal no pueden seguir frenando a la juventud afroEl artículoGuapi: donde navegar se convierte en liderazgo juvenil para transformar el Pacífico...</t>
         </is>
       </c>
     </row>
@@ -608,42 +608,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Prosperidad Social entregará transferencias a beneficiarios afectados por el terremoto sin verificación de condicionalidades y corresponsabilidades</t>
+          <t>De huir del conflicto a llevar agua segura y sostenible a las aulas: el liderazgo de Mabel Garcés en el Cauca</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prosperidad Social</t>
+          <t>Las2orillas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>gratuito</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>Violencia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Popayán</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://prosperidadsocial.gov.co/Noticias/prosperidad-social-entregara-transferencias-a-beneficiarios-afectados-por-el-terremoto-sin-verificacion-de-condicionalidades-y-corresponsabilidades/</t>
+          <t>https://www.las2orillas.co/de-huir-del-conflicto-a-llevar-agua-segura-y-sostenible-a-las-aulas-el-liderazgo-de-mabel-garces-en-el-cauca/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>El Gobierno nacional autorizó a Prosperidad Social a suspender temporalmente las verificaciones de corresponsabilidades que no puedan realizarse por las afectaciones del terremoto. La medida busca evitar que beneficiarios pierdan o retrasen sus...</t>
+          <t>Desplazada en su niñez por la violencia, esta joven llevó a un colegio de Puerto Tejada un sistema de agua limpia pensado y cuidado por la propia comunidaEl artículoDe huir del conflicto a llevar agua segura y sostenible a las aulas: el liderazgo de...</t>
         </is>
       </c>
     </row>

</xml_diff>